<commit_message>
Label renaming & incorporate stock-tail interpolation as part of pre-processing
</commit_message>
<xml_diff>
--- a/IMAGE-Mat/input/vehicles/data_raw/lifetimes_years.xlsx
+++ b/IMAGE-Mat/input/vehicles/data_raw/lifetimes_years.xlsx
@@ -1,79 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23426"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\surfdrive\Paper_5\Vehicle_Material_Model_Dynamic_SSP2020\vehicle_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\surfdrive - Sebastiaan Deetman@surfdrive.surf.nl\Github\Image\image-materials\IMAGE-Mat\input\vehicles\data_raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{62E8AE5D-1C37-48C5-A7AD-4453199E5AB0}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CDFEA44-639B-416B-90C1-213883B79C58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11385"/>
+    <workbookView xWindow="7200" yWindow="255" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="lifetimes_years" sheetId="1" r:id="rId1"/>
     <sheet name="car lifetime" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="26">
   <si>
-    <t>air_pas</t>
-  </si>
-  <si>
-    <t>air_freight</t>
-  </si>
-  <si>
-    <t>rail_reg</t>
-  </si>
-  <si>
-    <t>rail_hst</t>
-  </si>
-  <si>
-    <t>rail_freight</t>
-  </si>
-  <si>
-    <t>sea_shipping_small</t>
-  </si>
-  <si>
-    <t>sea_shipping_med</t>
-  </si>
-  <si>
-    <t>sea_shipping_large</t>
-  </si>
-  <si>
-    <t>sea_shipping_vl</t>
-  </si>
-  <si>
-    <t>LCV</t>
-  </si>
-  <si>
-    <t>MFT</t>
-  </si>
-  <si>
-    <t>HFT</t>
-  </si>
-  <si>
-    <t>midi_bus</t>
-  </si>
-  <si>
-    <t>reg_bus</t>
-  </si>
-  <si>
-    <t>inland_shipping</t>
-  </si>
-  <si>
-    <t>bicycle</t>
-  </si>
-  <si>
-    <t>car</t>
-  </si>
-  <si>
     <t>type</t>
   </si>
   <si>
@@ -99,12 +48,63 @@
   </si>
   <si>
     <t>Deetman et al. 2018</t>
+  </si>
+  <si>
+    <t>Planes</t>
+  </si>
+  <si>
+    <t>Freight Planes</t>
+  </si>
+  <si>
+    <t>Trains</t>
+  </si>
+  <si>
+    <t>High Speed Trains</t>
+  </si>
+  <si>
+    <t>Freight Trains</t>
+  </si>
+  <si>
+    <t>Small Ships</t>
+  </si>
+  <si>
+    <t>Medium Ships</t>
+  </si>
+  <si>
+    <t>Large Ships</t>
+  </si>
+  <si>
+    <t>Very Large Ships</t>
+  </si>
+  <si>
+    <t>Light Commercial Vehicles</t>
+  </si>
+  <si>
+    <t>Midi Buses</t>
+  </si>
+  <si>
+    <t>Inland Ships</t>
+  </si>
+  <si>
+    <t>Bikes</t>
+  </si>
+  <si>
+    <t>Cars</t>
+  </si>
+  <si>
+    <t>Regular Buses</t>
+  </si>
+  <si>
+    <t>Medium Freight Trucks</t>
+  </si>
+  <si>
+    <t>Heavy Freight Trucks</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -939,122 +939,122 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:T16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="C1" t="s">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D1" t="s">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="E1" t="s">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="F1" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="G1" t="s">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="H1" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="I1" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="J1" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="K1" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="L1" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="M1" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="N1" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="O1" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="P1" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="Q1" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="R1" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="G2" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="H2" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="I2" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="J2" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="K2" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="L2" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="N2" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="O2" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="P2" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="Q2" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="R2" t="s">
-        <v>19</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="B3">
         <v>20</v>
@@ -1110,7 +1110,7 @@
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="B4">
         <v>0.28100000000000003</v>
@@ -1166,7 +1166,7 @@
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -1223,7 +1223,7 @@
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -1299,24 +1299,24 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="D2" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>